<commit_message>
fixed issue with PFBS data missing from analysis
</commit_message>
<xml_diff>
--- a/data_input/Studies for time weighted average serum determination.xlsx
+++ b/data_input/Studies for time weighted average serum determination.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://oehhacloud-my.sharepoint.com/personal/scott_coffin_oehha_ca_gov/Documents/R_new/PFHpA/input/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://oehhacloud-my.sharepoint.com/personal/scott_coffin_oehha_ca_gov/Documents/R_new/Rat_TTR_PFAS_QSAR_Docking/data_input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E5A3DFD-22C0-44B7-B2C3-F819A306DC7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{6E5A3DFD-22C0-44B7-B2C3-F819A306DC7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6ABE660E-314A-4B0F-B837-41B2BC63F095}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-109" yWindow="-109" windowWidth="26301" windowHeight="14169" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="834" uniqueCount="155">
   <si>
     <t>Compound administered</t>
   </si>
@@ -678,25 +678,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -844,7 +832,13 @@
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CEBF3643-3ADA-4959-9FCE-DC410D8D8942}" name="Table1" displayName="Table1" ref="A1:AM33" totalsRowShown="0" headerRowDxfId="40" dataDxfId="39">
-  <autoFilter ref="A1:AM33" xr:uid="{CEBF3643-3ADA-4959-9FCE-DC410D8D8942}"/>
+  <autoFilter ref="A1:AM33" xr:uid="{CEBF3643-3ADA-4959-9FCE-DC410D8D8942}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="PFBS"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:AM31">
     <sortCondition ref="D1:D31"/>
   </sortState>
@@ -900,9 +894,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -940,7 +934,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1046,7 +1040,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1188,7 +1182,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1197,40 +1191,40 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AM33"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.3" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="29.5703125" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="43.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.625" customWidth="1"/>
+    <col min="3" max="3" width="19.25" customWidth="1"/>
+    <col min="4" max="4" width="43.625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19" customWidth="1"/>
-    <col min="6" max="6" width="37.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="37.75" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="7" customWidth="1"/>
-    <col min="8" max="8" width="103.42578125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="13" width="11.7109375" customWidth="1"/>
-    <col min="14" max="14" width="11.5703125" customWidth="1"/>
-    <col min="15" max="15" width="10.28515625" customWidth="1"/>
+    <col min="8" max="8" width="103.375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.75" bestFit="1" customWidth="1"/>
+    <col min="10" max="13" width="11.75" customWidth="1"/>
+    <col min="14" max="14" width="11.625" customWidth="1"/>
+    <col min="15" max="15" width="10.25" customWidth="1"/>
     <col min="16" max="16" width="20" customWidth="1"/>
-    <col min="17" max="18" width="12.5703125" customWidth="1"/>
-    <col min="19" max="22" width="13.140625" customWidth="1"/>
-    <col min="23" max="23" width="12.85546875" customWidth="1"/>
-    <col min="24" max="24" width="18.7109375" customWidth="1"/>
-    <col min="25" max="25" width="141.28515625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="18.7109375" customWidth="1"/>
-    <col min="27" max="30" width="17.140625" customWidth="1"/>
-    <col min="31" max="31" width="16.7109375" customWidth="1"/>
-    <col min="32" max="32" width="25.42578125" customWidth="1"/>
-    <col min="33" max="33" width="20.7109375" customWidth="1"/>
-    <col min="34" max="34" width="43.7109375" bestFit="1" customWidth="1"/>
-    <col min="35" max="36" width="28.7109375" customWidth="1"/>
-    <col min="37" max="37" width="14.85546875" customWidth="1"/>
-    <col min="38" max="38" width="23.140625" customWidth="1"/>
-    <col min="39" max="39" width="26.5703125" customWidth="1"/>
-    <col min="40" max="40" width="27.28515625" customWidth="1"/>
+    <col min="17" max="18" width="12.625" customWidth="1"/>
+    <col min="19" max="22" width="13.125" customWidth="1"/>
+    <col min="23" max="23" width="12.875" customWidth="1"/>
+    <col min="24" max="24" width="18.75" customWidth="1"/>
+    <col min="25" max="25" width="141.25" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="18.75" customWidth="1"/>
+    <col min="27" max="30" width="17.125" customWidth="1"/>
+    <col min="31" max="31" width="16.75" customWidth="1"/>
+    <col min="32" max="32" width="25.375" customWidth="1"/>
+    <col min="33" max="33" width="20.75" customWidth="1"/>
+    <col min="34" max="34" width="43.75" bestFit="1" customWidth="1"/>
+    <col min="35" max="36" width="28.75" customWidth="1"/>
+    <col min="37" max="37" width="14.875" customWidth="1"/>
+    <col min="38" max="38" width="23.125" customWidth="1"/>
+    <col min="39" max="39" width="26.625" customWidth="1"/>
+    <col min="40" max="40" width="27.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:39" s="1" customFormat="1" ht="14.95" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>96</v>
       </c>
@@ -1349,7 +1343,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="2" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>135</v>
       </c>
@@ -1471,7 +1465,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="3" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>135</v>
       </c>
@@ -1593,29 +1587,29 @@
         <v>672</v>
       </c>
     </row>
-    <row r="4" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7" t="s">
+    <row r="4" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="C4" s="7">
+      <c r="C4" s="3">
         <v>386.04</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="3" t="s">
         <v>144</v>
       </c>
       <c r="I4" s="1">
@@ -1668,7 +1662,7 @@
       <c r="X4" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="Y4" s="6" t="s">
+      <c r="Y4" s="1" t="s">
         <v>111</v>
       </c>
       <c r="Z4" s="1" t="s">
@@ -1695,16 +1689,16 @@
       <c r="AG4" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="AH4" s="7" t="s">
+      <c r="AH4" s="3" t="s">
         <v>15</v>
       </c>
       <c r="AI4" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="AJ4" s="7" t="s">
+      <c r="AJ4" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="AK4" s="7" t="s">
+      <c r="AK4" s="3" t="s">
         <v>151</v>
       </c>
       <c r="AL4" s="1">
@@ -1715,29 +1709,29 @@
         <v>2160</v>
       </c>
     </row>
-    <row r="5" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7" t="s">
+    <row r="5" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="3">
         <v>386.04</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="3" t="s">
         <v>144</v>
       </c>
       <c r="I5" s="1">
@@ -1790,7 +1784,7 @@
       <c r="X5" s="1" t="s">
         <v>111</v>
       </c>
-      <c r="Y5" s="6" t="s">
+      <c r="Y5" s="1" t="s">
         <v>111</v>
       </c>
       <c r="Z5" s="1" t="s">
@@ -1817,16 +1811,16 @@
       <c r="AG5" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="AH5" s="7" t="s">
+      <c r="AH5" s="3" t="s">
         <v>15</v>
       </c>
       <c r="AI5" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="AJ5" s="7" t="s">
+      <c r="AJ5" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="AK5" s="7" t="s">
+      <c r="AK5" s="3" t="s">
         <v>151</v>
       </c>
       <c r="AL5" s="1">
@@ -1837,7 +1831,7 @@
         <v>2160</v>
       </c>
     </row>
-    <row r="6" spans="1:39" s="1" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:39" s="1" customFormat="1" ht="59.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>7</v>
       </c>
@@ -1960,7 +1954,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="7" spans="1:39" s="1" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:39" s="1" customFormat="1" ht="59.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>7</v>
       </c>
@@ -2066,7 +2060,7 @@
       <c r="AH7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="AI7" s="6" t="s">
+      <c r="AI7" s="1" t="s">
         <v>103</v>
       </c>
       <c r="AJ7" s="1" t="s">
@@ -2083,7 +2077,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="8" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>132</v>
       </c>
@@ -2185,7 +2179,7 @@
       <c r="AH8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="AI8" s="6" t="s">
+      <c r="AI8" s="1" t="s">
         <v>103</v>
       </c>
       <c r="AJ8" s="1" t="s">
@@ -2202,7 +2196,7 @@
         <v>2160</v>
       </c>
     </row>
-    <row r="9" spans="1:39" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:39" s="1" customFormat="1" ht="16.3" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -2325,7 +2319,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="10" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>133</v>
       </c>
@@ -2448,7 +2442,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="11" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>133</v>
       </c>
@@ -2571,7 +2565,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="12" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>7</v>
       </c>
@@ -2693,7 +2687,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="13" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>132</v>
       </c>
@@ -2792,10 +2786,10 @@
       <c r="AG13" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="AH13" s="6" t="s">
+      <c r="AH13" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="AI13" s="6" t="s">
+      <c r="AI13" s="1" t="s">
         <v>103</v>
       </c>
       <c r="AJ13" s="1" t="s">
@@ -2813,7 +2807,7 @@
         <v>1464</v>
       </c>
     </row>
-    <row r="14" spans="1:39" s="1" customFormat="1" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:39" s="1" customFormat="1" ht="32.299999999999997" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>7</v>
       </c>
@@ -2915,7 +2909,7 @@
       <c r="AG14" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="AH14" s="6" t="s">
+      <c r="AH14" s="1" t="s">
         <v>81</v>
       </c>
       <c r="AI14" s="2" t="s">
@@ -2935,7 +2929,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="15" spans="1:39" s="1" customFormat="1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:39" s="1" customFormat="1" ht="30.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>76</v>
       </c>
@@ -3057,7 +3051,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="16" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>132</v>
       </c>
@@ -3177,7 +3171,7 @@
         <v>17976</v>
       </c>
     </row>
-    <row r="17" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>132</v>
       </c>
@@ -3297,7 +3291,7 @@
         <v>17976</v>
       </c>
     </row>
-    <row r="18" spans="1:39" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:39" s="1" customFormat="1" ht="30.1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>133</v>
       </c>
@@ -3419,7 +3413,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="19" spans="1:39" s="1" customFormat="1" ht="30" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:39" s="1" customFormat="1" ht="30.1" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>133</v>
       </c>
@@ -3541,7 +3535,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="20" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>132</v>
       </c>
@@ -3660,7 +3654,7 @@
         <v>2208</v>
       </c>
     </row>
-    <row r="21" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>132</v>
       </c>
@@ -3779,7 +3773,7 @@
         <v>2208</v>
       </c>
     </row>
-    <row r="22" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:39" s="1" customFormat="1" ht="14.95" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>61</v>
       </c>
@@ -3834,22 +3828,22 @@
         <v>56</v>
       </c>
       <c r="R22" s="1">
+        <v>0</v>
+      </c>
+      <c r="S22" s="1">
         <v>0.09</v>
       </c>
-      <c r="S22" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="T22" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="U22" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="V22" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="W22" s="1" t="s">
-        <v>111</v>
+      <c r="T22" s="1">
+        <v>2.222</v>
+      </c>
+      <c r="U22" s="1">
+        <v>5.3659999999999997</v>
+      </c>
+      <c r="V22" s="1">
+        <v>12.43</v>
+      </c>
+      <c r="W22" s="1">
+        <v>43.16</v>
       </c>
       <c r="X22" s="1" t="s">
         <v>125</v>
@@ -3902,7 +3896,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="23" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:39" s="1" customFormat="1" ht="14.95" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>61</v>
       </c>
@@ -3957,22 +3951,22 @@
         <v>56</v>
       </c>
       <c r="R23" s="1">
-        <v>2.5000000000000001E-2</v>
-      </c>
-      <c r="S23" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="T23" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="U23" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="V23" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="W23" s="1" t="s">
-        <v>111</v>
+        <v>0</v>
+      </c>
+      <c r="S23" s="1">
+        <v>0.154</v>
+      </c>
+      <c r="T23" s="1">
+        <v>0.309</v>
+      </c>
+      <c r="U23" s="1">
+        <v>0.93100000000000005</v>
+      </c>
+      <c r="V23" s="1">
+        <v>8.1709999999999994</v>
+      </c>
+      <c r="W23" s="1">
+        <v>25.454999999999998</v>
       </c>
       <c r="X23" s="1" t="s">
         <v>125</v>
@@ -4025,7 +4019,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="24" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>134</v>
       </c>
@@ -4148,7 +4142,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="25" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>134</v>
       </c>
@@ -4164,7 +4158,7 @@
       <c r="E25" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F25" s="6" t="s">
+      <c r="F25" s="1" t="s">
         <v>39</v>
       </c>
       <c r="G25" s="1" t="s">
@@ -4271,7 +4265,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="26" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>132</v>
       </c>
@@ -4287,7 +4281,7 @@
       <c r="E26" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F26" s="6" t="s">
+      <c r="F26" s="1" t="s">
         <v>39</v>
       </c>
       <c r="G26" s="1" t="s">
@@ -4394,7 +4388,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="27" spans="1:39" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:39" s="1" customFormat="1" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>132</v>
       </c>
@@ -4500,7 +4494,7 @@
       <c r="AH27" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AI27" s="6" t="s">
+      <c r="AI27" s="1" t="s">
         <v>103</v>
       </c>
       <c r="AJ27" s="1" t="s">
@@ -4517,657 +4511,657 @@
         <v>672</v>
       </c>
     </row>
-    <row r="28" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A28" s="4" t="s">
+    <row r="28" spans="1:39" ht="14.95" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="B28" s="4" t="s">
+      <c r="B28" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="C28" s="4">
+      <c r="C28" s="3">
         <v>414.07</v>
       </c>
-      <c r="D28" s="4" t="s">
+      <c r="D28" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="E28" s="4" t="s">
+      <c r="E28" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="F28" s="4" t="s">
+      <c r="F28" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="G28" s="4" t="s">
+      <c r="G28" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="H28" s="4" t="s">
+      <c r="H28" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="I28" s="3">
+      <c r="I28" s="1">
         <v>0</v>
       </c>
-      <c r="J28" s="3">
+      <c r="J28" s="1">
         <v>6.25</v>
       </c>
-      <c r="K28" s="3">
+      <c r="K28" s="1">
         <v>12.5</v>
       </c>
-      <c r="L28" s="3">
+      <c r="L28" s="1">
         <v>25</v>
       </c>
-      <c r="M28" s="6">
+      <c r="M28" s="1">
         <v>50</v>
       </c>
-      <c r="N28" s="6">
+      <c r="N28" s="1">
         <v>100</v>
       </c>
-      <c r="O28" s="6">
-        <v>24</v>
-      </c>
-      <c r="P28" s="3">
+      <c r="O28" s="1">
+        <v>24</v>
+      </c>
+      <c r="P28" s="1">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="Q28" s="3">
+      <c r="Q28" s="1">
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="R28" s="6">
+      <c r="R28" s="1">
         <v>0</v>
       </c>
-      <c r="S28" s="6">
+      <c r="S28" s="1">
         <v>0.49099999999999999</v>
       </c>
-      <c r="T28" s="6">
+      <c r="T28" s="1">
         <v>1.153</v>
       </c>
-      <c r="U28" s="6">
+      <c r="U28" s="1">
         <v>2.96</v>
       </c>
-      <c r="V28" s="6">
+      <c r="V28" s="1">
         <v>9.3260000000000005</v>
       </c>
-      <c r="W28" s="6">
+      <c r="W28" s="1">
         <v>23.443999999999999</v>
       </c>
-      <c r="X28" s="6" t="s">
+      <c r="X28" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="Y28" s="7" t="s">
+      <c r="Y28" s="3" t="s">
         <v>149</v>
       </c>
-      <c r="Z28" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AA28" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AB28" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AC28" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD28" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AE28" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AF28" s="6">
+      <c r="Z28" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA28" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AB28" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AC28" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD28" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AE28" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AF28" s="1">
         <f t="shared" si="3"/>
         <v>696</v>
       </c>
-      <c r="AG28" s="6" t="s">
+      <c r="AG28" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="AH28" s="7" t="s">
+      <c r="AH28" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="AI28" s="6" t="s">
+      <c r="AI28" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="AJ28" s="7" t="s">
+      <c r="AJ28" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="AK28" s="7" t="s">
+      <c r="AK28" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="AL28" s="3">
+      <c r="AL28" s="1">
         <v>28</v>
       </c>
-      <c r="AM28" s="3">
+      <c r="AM28" s="1">
         <f t="shared" si="2"/>
         <v>672</v>
       </c>
     </row>
-    <row r="29" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A29" s="6" t="s">
+    <row r="29" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="B29" s="6" t="s">
+      <c r="B29" s="1" t="s">
         <v>145</v>
       </c>
-      <c r="C29" s="6">
+      <c r="C29" s="1">
         <v>414.07</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="1" t="s">
         <v>146</v>
       </c>
-      <c r="E29" s="6" t="s">
+      <c r="E29" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F29" s="6" t="s">
+      <c r="F29" s="1" t="s">
         <v>147</v>
       </c>
-      <c r="G29" s="6" t="s">
+      <c r="G29" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="H29" s="6" t="s">
+      <c r="H29" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="I29" s="3">
+      <c r="I29" s="1">
         <v>0</v>
       </c>
-      <c r="J29" s="6">
+      <c r="J29" s="1">
         <v>0.625</v>
       </c>
-      <c r="K29" s="6">
+      <c r="K29" s="1">
         <v>1.25</v>
       </c>
-      <c r="L29" s="6">
+      <c r="L29" s="1">
         <v>2.5</v>
       </c>
-      <c r="M29" s="6">
+      <c r="M29" s="1">
         <v>5</v>
       </c>
-      <c r="N29" s="6">
+      <c r="N29" s="1">
         <v>10</v>
       </c>
-      <c r="O29" s="6">
-        <v>24</v>
-      </c>
-      <c r="P29" s="3">
+      <c r="O29" s="1">
+        <v>24</v>
+      </c>
+      <c r="P29" s="1">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="Q29" s="3">
+      <c r="Q29" s="1">
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="R29" s="6">
+      <c r="R29" s="1">
         <v>9.8000000000000004E-2</v>
       </c>
-      <c r="S29" s="6">
+      <c r="S29" s="1">
         <v>50.69</v>
       </c>
-      <c r="T29" s="6">
+      <c r="T29" s="1">
         <v>73.48</v>
       </c>
-      <c r="U29" s="6">
+      <c r="U29" s="1">
         <v>95.43</v>
       </c>
-      <c r="V29" s="6">
+      <c r="V29" s="1">
         <v>110.72</v>
       </c>
-      <c r="W29" s="6">
+      <c r="W29" s="1">
         <v>148.57</v>
       </c>
-      <c r="X29" s="6" t="s">
+      <c r="X29" s="1" t="s">
         <v>125</v>
       </c>
-      <c r="Y29" s="6" t="s">
+      <c r="Y29" s="1" t="s">
         <v>150</v>
       </c>
-      <c r="Z29" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AA29" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AB29" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AC29" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD29" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AE29" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AF29" s="6">
+      <c r="Z29" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA29" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AB29" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AC29" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD29" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AE29" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AF29" s="1">
         <f t="shared" si="3"/>
         <v>696</v>
       </c>
-      <c r="AG29" s="6" t="s">
+      <c r="AG29" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="AH29" s="6" t="s">
+      <c r="AH29" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="AI29" s="6" t="s">
+      <c r="AI29" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="AJ29" s="6" t="s">
+      <c r="AJ29" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="AK29" s="6" t="s">
+      <c r="AK29" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="AL29" s="3">
+      <c r="AL29" s="1">
         <v>28</v>
       </c>
-      <c r="AM29" s="3">
+      <c r="AM29" s="1">
         <f t="shared" si="2"/>
         <v>672</v>
       </c>
     </row>
-    <row r="30" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A30" s="6" t="s">
+    <row r="30" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="B30" s="6" t="s">
+      <c r="B30" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C30" s="6">
+      <c r="C30" s="1">
         <v>364.06</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E30" s="6" t="s">
+      <c r="E30" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F30" s="6" t="s">
+      <c r="F30" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="G30" s="6" t="s">
+      <c r="G30" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="H30" s="6" t="s">
+      <c r="H30" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="I30" s="3">
+      <c r="I30" s="1">
         <v>0</v>
       </c>
-      <c r="J30" s="3">
+      <c r="J30" s="1">
         <v>31.25</v>
       </c>
-      <c r="K30" s="3">
+      <c r="K30" s="1">
         <v>62.5</v>
       </c>
-      <c r="L30" s="3">
+      <c r="L30" s="1">
         <v>125</v>
       </c>
-      <c r="M30" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="N30" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="O30" s="6">
-        <v>24</v>
-      </c>
-      <c r="P30" s="3">
+      <c r="M30" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="N30" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="O30" s="1">
+        <v>24</v>
+      </c>
+      <c r="P30" s="1">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="Q30" s="3">
+      <c r="Q30" s="1">
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="R30" s="3">
+      <c r="R30" s="1">
         <v>0.8</v>
       </c>
-      <c r="S30" s="3">
+      <c r="S30" s="1">
         <v>63.5</v>
       </c>
-      <c r="T30" s="3">
+      <c r="T30" s="1">
         <v>93.2</v>
       </c>
-      <c r="U30" s="3">
+      <c r="U30" s="1">
         <v>139.19999999999999</v>
       </c>
-      <c r="V30" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="W30" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="X30" s="3" t="s">
+      <c r="V30" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="W30" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="X30" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="Y30" s="6" t="s">
+      <c r="Y30" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="Z30" s="6">
+      <c r="Z30" s="1">
         <v>0.5</v>
       </c>
-      <c r="AA30" s="6">
+      <c r="AA30" s="1">
         <v>36.299999999999997</v>
       </c>
-      <c r="AB30" s="6">
+      <c r="AB30" s="1">
         <v>36.299999999999997</v>
       </c>
-      <c r="AC30" s="6">
+      <c r="AC30" s="1">
         <v>60.4</v>
       </c>
-      <c r="AD30" s="6"/>
-      <c r="AE30" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AF30" s="6">
+      <c r="AD30" s="1"/>
+      <c r="AE30" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AF30" s="1">
         <f t="shared" si="3"/>
         <v>696</v>
       </c>
-      <c r="AG30" s="6" t="s">
+      <c r="AG30" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="AH30" s="6" t="s">
+      <c r="AH30" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="AI30" s="6" t="s">
+      <c r="AI30" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="AJ30" s="6" t="s">
+      <c r="AJ30" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="AK30" s="6" t="s">
+      <c r="AK30" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="AL30" s="3">
+      <c r="AL30" s="1">
         <v>28</v>
       </c>
-      <c r="AM30" s="3">
+      <c r="AM30" s="1">
         <f t="shared" si="2"/>
         <v>672</v>
       </c>
     </row>
-    <row r="31" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A31" s="3" t="s">
+    <row r="31" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B31" s="3" t="s">
+      <c r="B31" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C31" s="3">
+      <c r="C31" s="1">
         <v>314.05</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="E31" s="3" t="s">
+      <c r="E31" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F31" s="3" t="s">
+      <c r="F31" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="G31" s="3" t="s">
+      <c r="G31" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="H31" s="3" t="s">
+      <c r="H31" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="I31" s="3">
+      <c r="I31" s="1">
         <v>0</v>
       </c>
-      <c r="J31" s="3">
+      <c r="J31" s="1">
         <v>31.25</v>
       </c>
-      <c r="K31" s="3">
+      <c r="K31" s="1">
         <v>62.5</v>
       </c>
-      <c r="L31" s="3">
+      <c r="L31" s="1">
         <v>125</v>
       </c>
-      <c r="M31" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="N31" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="O31" s="6">
-        <v>24</v>
-      </c>
-      <c r="P31" s="3">
+      <c r="M31" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="N31" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="O31" s="1">
+        <v>24</v>
+      </c>
+      <c r="P31" s="1">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="Q31" s="3">
+      <c r="Q31" s="1">
         <f t="shared" si="1"/>
         <v>28</v>
       </c>
-      <c r="R31" s="3">
+      <c r="R31" s="1">
         <v>0</v>
       </c>
-      <c r="S31" s="3">
+      <c r="S31" s="1">
         <v>1.3</v>
       </c>
-      <c r="T31" s="3">
+      <c r="T31" s="1">
         <v>3.1</v>
       </c>
-      <c r="U31" s="3">
+      <c r="U31" s="1">
         <v>4.5</v>
       </c>
-      <c r="V31" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="W31" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="X31" s="3" t="s">
+      <c r="V31" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="W31" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="X31" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="Y31" s="5" t="s">
+      <c r="Y31" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="Z31" s="6">
+      <c r="Z31" s="1">
         <v>0.2</v>
       </c>
-      <c r="AA31" s="6">
+      <c r="AA31" s="1">
         <v>0.9</v>
       </c>
-      <c r="AB31" s="6">
+      <c r="AB31" s="1">
         <v>0.9</v>
       </c>
-      <c r="AC31" s="6">
+      <c r="AC31" s="1">
         <v>2.7</v>
       </c>
-      <c r="AD31" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AE31" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AF31" s="6">
+      <c r="AD31" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AE31" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AF31" s="1">
         <f t="shared" si="3"/>
         <v>696</v>
       </c>
-      <c r="AG31" s="6" t="s">
+      <c r="AG31" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="AH31" s="6" t="s">
+      <c r="AH31" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="AI31" s="6" t="s">
+      <c r="AI31" s="1" t="s">
         <v>102</v>
       </c>
-      <c r="AJ31" s="6" t="s">
+      <c r="AJ31" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="AK31" s="6" t="s">
+      <c r="AK31" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="AL31" s="3">
+      <c r="AL31" s="1">
         <v>28</v>
       </c>
-      <c r="AM31" s="3">
+      <c r="AM31" s="1">
         <f t="shared" si="2"/>
         <v>672</v>
       </c>
     </row>
-    <row r="32" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A32" s="6" t="s">
+    <row r="32" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B32" s="6" t="s">
+      <c r="B32" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C32" s="2">
         <v>231.07</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="1" t="s">
         <v>152</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E32" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F32" s="6" t="s">
+      <c r="F32" s="1" t="s">
         <v>143</v>
       </c>
-      <c r="G32" s="6" t="s">
+      <c r="G32" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="H32" s="6" t="s">
+      <c r="H32" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="I32" s="6">
+      <c r="I32" s="1">
         <v>0</v>
       </c>
-      <c r="J32" s="6">
+      <c r="J32" s="1">
         <v>35</v>
       </c>
-      <c r="K32" s="6">
+      <c r="K32" s="1">
         <v>175</v>
       </c>
-      <c r="L32" s="6">
+      <c r="L32" s="1">
         <v>350</v>
       </c>
-      <c r="M32" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="N32" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="O32" s="6">
-        <v>24</v>
-      </c>
-      <c r="P32" s="6">
+      <c r="M32" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="N32" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="O32" s="1">
+        <v>24</v>
+      </c>
+      <c r="P32" s="1">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="Q32" s="6">
+      <c r="Q32" s="1">
         <f t="shared" si="1"/>
         <v>17</v>
       </c>
-      <c r="R32" s="6">
+      <c r="R32" s="1">
         <v>2E-3</v>
       </c>
-      <c r="S32" s="6">
+      <c r="S32" s="1">
         <v>3.78</v>
       </c>
-      <c r="T32" s="6">
+      <c r="T32" s="1">
         <v>4.4400000000000004</v>
       </c>
-      <c r="U32" s="6">
+      <c r="U32" s="1">
         <v>2.4900000000000002</v>
       </c>
-      <c r="V32" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="W32" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="X32" s="6" t="s">
+      <c r="V32" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="W32" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="X32" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="Y32" s="6"/>
-      <c r="Z32" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AA32" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AB32" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AC32" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AD32" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AE32" s="6" t="s">
-        <v>111</v>
-      </c>
-      <c r="AF32" s="6">
+      <c r="Y32" s="1"/>
+      <c r="Z32" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AA32" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AB32" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AC32" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AD32" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AE32" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="AF32" s="1">
         <f t="shared" si="3"/>
         <v>432</v>
       </c>
-      <c r="AG32" s="6" t="s">
+      <c r="AG32" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="AH32" s="6" t="s">
+      <c r="AH32" s="1" t="s">
         <v>153</v>
       </c>
-      <c r="AI32" s="6" t="s">
+      <c r="AI32" s="1" t="s">
         <v>103</v>
       </c>
-      <c r="AJ32" s="6" t="s">
+      <c r="AJ32" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="AK32" s="6" t="s">
+      <c r="AK32" s="1" t="s">
         <v>154</v>
       </c>
-      <c r="AL32" s="6">
+      <c r="AL32" s="1">
         <v>17</v>
       </c>
-      <c r="AM32" s="6">
+      <c r="AM32" s="1">
         <f t="shared" si="2"/>
         <v>408</v>
       </c>
     </row>
-    <row r="33" spans="1:39" x14ac:dyDescent="0.25">
-      <c r="A33" s="6"/>
-      <c r="B33" s="6"/>
-      <c r="C33" s="6"/>
-      <c r="D33" s="6"/>
-      <c r="E33" s="6"/>
-      <c r="F33" s="6"/>
-      <c r="G33" s="6"/>
-      <c r="H33" s="6"/>
-      <c r="I33" s="6"/>
-      <c r="J33" s="6"/>
-      <c r="K33" s="6"/>
-      <c r="L33" s="6"/>
-      <c r="M33" s="6"/>
-      <c r="N33" s="6"/>
-      <c r="O33" s="6"/>
-      <c r="P33" s="6"/>
-      <c r="Q33" s="6"/>
-      <c r="R33" s="6"/>
-      <c r="S33" s="6"/>
-      <c r="T33" s="6"/>
-      <c r="U33" s="6"/>
-      <c r="V33" s="6"/>
-      <c r="W33" s="6"/>
-      <c r="X33" s="6"/>
-      <c r="Y33" s="6"/>
-      <c r="Z33" s="6"/>
-      <c r="AA33" s="6"/>
-      <c r="AB33" s="6"/>
-      <c r="AC33" s="6"/>
-      <c r="AD33" s="6"/>
-      <c r="AE33" s="6"/>
-      <c r="AF33" s="6"/>
-      <c r="AG33" s="6"/>
-      <c r="AH33" s="6"/>
-      <c r="AI33" s="6"/>
-      <c r="AJ33" s="6"/>
-      <c r="AK33" s="6"/>
-      <c r="AL33" s="6"/>
-      <c r="AM33" s="6"/>
+    <row r="33" spans="1:39" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1"/>
+      <c r="O33" s="1"/>
+      <c r="P33" s="1"/>
+      <c r="Q33" s="1"/>
+      <c r="R33" s="1"/>
+      <c r="S33" s="1"/>
+      <c r="T33" s="1"/>
+      <c r="U33" s="1"/>
+      <c r="V33" s="1"/>
+      <c r="W33" s="1"/>
+      <c r="X33" s="1"/>
+      <c r="Y33" s="1"/>
+      <c r="Z33" s="1"/>
+      <c r="AA33" s="1"/>
+      <c r="AB33" s="1"/>
+      <c r="AC33" s="1"/>
+      <c r="AD33" s="1"/>
+      <c r="AE33" s="1"/>
+      <c r="AF33" s="1"/>
+      <c r="AG33" s="1"/>
+      <c r="AH33" s="1"/>
+      <c r="AI33" s="1"/>
+      <c r="AJ33" s="1"/>
+      <c r="AK33" s="1"/>
+      <c r="AL33" s="1"/>
+      <c r="AM33" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>